<commit_message>
Comenzi Miyawaki: oferta Mizil (4 din 12 specii), speciile lipsă mutate la Pepiniera Silvică Agigea și Doi Cocoși, cerere de ofertă Agigea, starea comenzilor în generator
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/cereri/cerere-oferta-pepiniera-doi-cocosi-srl.xlsx
+++ b/resurse/oferte/cereri/cerere-oferta-pepiniera-doi-cocosi-srl.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -624,34 +624,63 @@
       <c r="H12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr"/>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Cireș sălbatic</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Prunus avium</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1–2 ani, 30–80 cm, rădăcină nudă sau ghiveci 1–2 l</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5">
+        <f>D13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7">
-        <f>SUM(D11:D12)</f>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7">
+        <f>SUM(D11:D13)</f>
         <v/>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7">
-        <f>SUM(G11:G12)</f>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7">
+        <f>SUM(G11:G13)</f>
         <v/>
       </c>
-      <c r="H13" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Vă rugăm să precizați: costul transportului la Crucea sau adresa de ridicare, termenul de valabilitate al ofertei, dacă puteți rezerva cantitățile până la confirmare, și eventualele specii pe care nu le aveți (cu propuneri de înlocuire).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Vă mulțumim.</t>
         </is>
@@ -661,8 +690,8 @@
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A15:H15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>